<commit_message>
Vorbereitung auf Charakter Texte
</commit_message>
<xml_diff>
--- a/Dokumente/Dhampir-Datenbank.xlsx
+++ b/Dokumente/Dhampir-Datenbank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dokumente\1. Projekte\Dhampir\Dokumente\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE08B90F-A66D-4ED8-A7BF-9D7B0CD6A1E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{717BDA4F-5029-455D-B5BC-DB8843161AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Bruderschaft der Dhampire</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Gegnertypen (9)</t>
   </si>
   <si>
-    <t>Basis der Ritter der Nacht</t>
-  </si>
-  <si>
     <t>Die Ritter der Nacht</t>
   </si>
   <si>
@@ -303,8 +300,196 @@
     </r>
   </si>
   <si>
-    <t>Basim überlebte seine Kindheit durch Schlauheit und das, was andere wegwarfen. Tagsüber leerte er mit seiner Freundin Nihal den Leuten dir Taschen, des nachts quälte ein furchterregender Dschinn, den Schlaf des jungen Straßendiebes.
-Ehrgeizig und von dem Wunsch getrieben, der Gerechtigkeit zu dienen, sehnte sich Basim danach, ein Verborgener zu werden. Je näher er jedoch seinem Traum kam, desto näher kam auch sein Nachtmahr.</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sebastian, die Fledermaus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Schon als Kleinkind fand er (laut seiner Eltern) eine Babyfledermaus, die er aufzog und die seit jeher ein festes Band der Verbundenheit eint. Aufgrund seiner Gabe die er im Prolog entdeckte, kann er mit seinem Begleiter kommunizieren, wobei ihn "Sebi" beim observieren der Missionsstandorte hilft, ihn aber auch in mancher brenzliger Situation, vor den Feinden rettet. Daniel und seinem Haustier eint dabei das verlangen herauszufinden woher und was Sie sind, den auch Sebi zeigt eine Veränderung wen er Blut aufnimmt, wie man beobachten konnte. So konnte man erkennen das hinter seiner putzigen Gestalt sich ein besonderes Geheimnis verbirgt.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Akt 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Eingesperrt in einer Tropfsteinhöhle kann nur er seine Kumpanen und besten Freund retten, die Fledermaus "Sebastian". Zeige dein ganzes Können in dieser besonderen Gestalt. Seine ersten Auswegsversuche waren dabei zwar armselig, aber er gibt immer Erfolge, wen man an Sie glaubt.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Jessica, die dunkle Werwolfbraut</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Im Kindergarten lernte Sie den etwas verschlossenen Daniel kennen, der immer schon etwas anders war. Obwohl nur ein paar Monate jünger als Sie, entwickelt sich schon da ein "Große Schwester" empfinden zu ihm. Als Sie schließlich herausfand, das Sie zu einem Werwolfclan (ihr Vater ist der Werlord der Region) gehört und als deren Erbe ergoren ist, wurde Sie angewissen ihren besten Freund aus zuspionieren und notfalls umzubringen, wen er zur Gefahr für die "Anderwelt" (Welt der Mischwesen) werden würde, wie andere seiner Wesensart vor ihm. Um dies zu verhindern und ihn zu beschützen, schafft Sie mit ihm aber ein Team zusammen, was mit ihren unterschiedlichen Stärken, diese Aufgabe abwenden soll und Daniel in eine Richtung die ihm zum Beschützer der Anderwelt macht.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Akt 16</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Nach Daniels Rückkehr im Rheinland kommt der Werwolfclan zur Entscheidung, sein Leben als Opfer für ihren Wergott zu opfern. Jessica entscheidet daraufhin, den Clan zu verlassen und gemeinsam mit den Rittern den Sie angehört, dieses Opfer zu verhindern, um weiter mit Daniel nach den Fragen der Herkunft, Aufgabe und Zukunftsherausforderungen zu suchen.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Utz, der Mediziner und grüne Hexer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+A
+Akt 1: </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Thutmosis, der Ägyptologe und dunkle Hexer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+A
+Akt 3:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Jan, der Geschichtsstudent und Púcca</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+A
+Akt 6:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sabrina, die Stadtbeamtin und Sirene</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+A
+Akt 12:</t>
+    </r>
   </si>
   <si>
     <r>
@@ -349,100 +534,12 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>: Das letzte was er von Akt 13 noch wahr nahm, das ihn auf seinem Heimweg ein kalter Lufthauch und die Gier nach Blut erheilte, nun findet er sich in einem alten Gemäuer eines Gebäudes des Balkan wieder. Seiner Versuche aus diesem Labyrinth waren bislang nich von Erfolg gekrönt und machen ihn nur hoffnungsloser. Gerade hatte man sich als Team zusammengefunden, aber nun war er hier allein mit seinen Erzfeinden, mit denen er wenigstens wie in einem Art Bootcamp trainieren konnte.</t>
+      <t>: Das letzte was er von Akt 13 noch wahr nahm, das ihn auf seinem Heimweg ein kalter Lufthauch und die Gier nach Blut ereilte, nun findet er sich in einem alten Gemäuer eines Gebäudes des Balkan wieder. Seiner Versuche aus diesem Labyrinth waren bislang nich von Erfolg gekrönt und machen ihn nur hoffnungsloser. Gerade hatte man sich als Team zusammengefunden, aber nun war er hier allein mit seinen Erzfeinden, mit denen er wenigstens wie in einem Art Bootcamp trainieren konnte.</t>
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Sebastian, die Fledermaus</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Schon als Kleinkind fand er (laut seiner Eltern) eine Babyfledermaus, die er aufzog und die seit jeher ein festes Band der Verbundenheit eint. Aufgrund seiner Gabe die er im Prolog entdeckte, kann er mit seinem Begleiter kommunizieren, wobei ihn "Sebi" beim observieren der Missionsstandorte hilft, ihn aber auch in mancher brenzliger Situation, vor den Feinden rettet. Daniel und seinem Haustier eint dabei das verlangen herauszufinden woher und was Sie sind, den auch Sebi zeigt eine Veränderung wen er Blut aufnimmt, wie man beobachten konnte. So konnte man erkennen das hinter seiner putzigen Gestalt sich ein besonderes Geheimnis verbirgt.
+    <t xml:space="preserve">Basis der Ritter der Nacht
 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Akt 5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: Eingesperrt in einer Tropfsteinhöhle kann nur er seine Kumpanen und besten Freund retten, die Fledermaus "Sebastian". Zeige dein ganzes Können in dieser besonderen Gestalt. Seine ersten Auswegsversuche waren dabei zwar armselig, aber er gibt immer Erfolge, wen man an Sie glaubt.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Jessica, die dunkle Werwolfbraut</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Im Kindergarten lernte Sie den etwas verschlossenen Daniel kennen, der immer schon etwas anders war. Obwohl nur ein paar Monate jünger als Sie, entwickelt sich schon da ein "Große Schwester" empfinden zu ihm. Als Sie schließlich herausfand, das Sie zu einem Werwolfclan (ihr Vater ist der Werlord der Region) gehört und als deren Erbe ergoren ist, wurde Sie angewissen ihren besten Freund aus zuspionieren und notfalls umzubringen, wen er zur Gefahr für die "Anderwelt" (Welt der Mischwesen) werden würde, wie andere seiner Wesensart vor ihm. Um dies zu verhindern und ihn zu beschützen, schafft Sie mit ihm aber ein Team zusammen, was mit ihren unterschiedlichen Stärken, diese Aufgabe abwenden soll und Daniel in eine Richtung die ihm zum Beschützer der Anderwelt macht.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Akt 16</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: Nach Daniels Rückkehr im Rheinland kommt der Werwolfclan zur Entscheidung, sein Leben als Opfer für ihren Wergott zu opfern. Jessica entscheidet daraufhin, den Clan zu verlassen und gemeinsam mit den Rittern den Sie angehört, dieses Opfer zu verhindern, um weiter mit Daniel nach den Fragen der Herkunft, Aufgabe und Zukunftsherausforderungen zu suchen.</t>
-    </r>
   </si>
 </sst>
 </file>
@@ -669,7 +766,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -736,6 +833,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1026,7 +1129,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="229.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="25.140625" style="2" bestFit="1" customWidth="1"/>
@@ -1083,7 +1186,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>4</v>
@@ -1112,11 +1215,11 @@
     </row>
     <row r="5" spans="1:21" ht="166.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15"/>
-      <c r="B5" s="9" t="s">
-        <v>7</v>
+      <c r="B5" s="23" t="s">
+        <v>18</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -1139,9 +1242,9 @@
     </row>
     <row r="6" spans="1:21" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
-      <c r="B6" s="10"/>
+      <c r="B6" s="24"/>
       <c r="C6" s="20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
@@ -1164,9 +1267,9 @@
     </row>
     <row r="7" spans="1:21" ht="90.75" x14ac:dyDescent="0.25">
       <c r="A7" s="16"/>
-      <c r="B7" s="10"/>
+      <c r="B7" s="24"/>
       <c r="C7" s="20" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
@@ -1189,9 +1292,9 @@
     </row>
     <row r="8" spans="1:21" ht="90.75" x14ac:dyDescent="0.25">
       <c r="A8" s="16"/>
-      <c r="B8" s="10"/>
+      <c r="B8" s="24"/>
       <c r="C8" s="20" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
@@ -1214,9 +1317,9 @@
     </row>
     <row r="9" spans="1:21" ht="105.75" x14ac:dyDescent="0.25">
       <c r="A9" s="16"/>
-      <c r="B9" s="10"/>
+      <c r="B9" s="24"/>
       <c r="C9" s="20" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
@@ -1237,10 +1340,12 @@
       <c r="T9" s="10"/>
       <c r="U9" s="5"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="20"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="20" t="s">
+        <v>13</v>
+      </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -1260,10 +1365,12 @@
       <c r="T10" s="10"/>
       <c r="U10" s="5"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="20"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="20" t="s">
+        <v>14</v>
+      </c>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -1283,10 +1390,12 @@
       <c r="T11" s="10"/>
       <c r="U11" s="5"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="20"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="20" t="s">
+        <v>15</v>
+      </c>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -1306,10 +1415,12 @@
       <c r="T12" s="10"/>
       <c r="U12" s="5"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="20"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="20" t="s">
+        <v>16</v>
+      </c>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -1470,7 +1581,7 @@
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="16"/>
       <c r="B20" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -2186,9 +2297,7 @@
     </row>
     <row r="51" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="52" spans="1:21" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C52" s="22" t="s">
-        <v>12</v>
-      </c>
+      <c r="C52" s="22"/>
       <c r="D52" s="18"/>
       <c r="E52" s="18"/>
       <c r="F52" s="18"/>
@@ -2328,9 +2437,10 @@
       <c r="J65" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="C52:C53"/>
+    <mergeCell ref="B5:B13"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>